<commit_message>
roadmap: ajoute onboarding conversationnel + Fil A+B + routines (post-tests)
Décisions validées avec user, à implémenter après tests Barbara :
- Onboarding conversationnel 4 questions (P0, gros refactor)
- Fil dans Journal : Yova messagère + moments clés (pas d'onglet)
- Détection de routines (groupement auto de tâches récurrentes)
- SMS hebdo opt-in au partenaire non-installé

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ROADMAP.xlsx
+++ b/docs/ROADMAP.xlsx
@@ -921,7 +921,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F9"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
     <col min="2" max="2" width="40.83203125" customWidth="1"/>
@@ -956,19 +956,19 @@
         <v>2.1</v>
       </c>
       <c r="B2" t="str">
-        <v>Wire up /api/ai/anticipate</v>
+        <v>Onboarding conversationnel (4 questions)</v>
       </c>
       <c r="C2" t="str">
-        <v>Endpoint d'anticipation proactive (tâches à venir, rappels). Route existe côté serveur. Brancher au dashboard : appel hebdomadaire qui affiche une carte "Yova anticipe : X tâches vont arriver cette semaine".</v>
+        <v>Remplacer les 4-5 écrans actuels (équipements + famille + baseline + catalogue + thinking) par une conversation vocale/texte de 3 min : Yova pose 4 questions (composition foyer, qui fait quoi, équipements, projet à venir). Claude génère famille + 15 tâches + pack projet éventuel en une passe via route /api/ai/onboarding-bootstrap. Plus naturel, plus rapide, profil pré-rempli dès le départ.</v>
       </c>
       <c r="D2" t="str">
         <v>À faire</v>
       </c>
       <c r="E2" t="str">
-        <v>P1</v>
+        <v>P0</v>
       </c>
       <c r="F2" t="str">
-        <v>User insistait dessus</v>
+        <v>Post-tests Barbara · gros refactor</v>
       </c>
     </row>
     <row r="3">
@@ -976,19 +976,19 @@
         <v>2.2</v>
       </c>
       <c r="B3" t="str">
-        <v>Wire up /api/ai/insights</v>
+        <v>Fil dans Journal (option A + B)</v>
       </c>
       <c r="C3" t="str">
-        <v>Insights IA hebdomadaires (version Premium de ce que DashboardFree fait côté client). Brancher au dashboard derrière gate Premium.</v>
+        <v>Pas d'onglet Fil dédié. Intégrer la reconnaissance dans le Journal : A. Yova messagère — quand Barbara complète une tâche, Yova l'annonce dans ton journal, tu réponds par ❤️/message libre → transmis à Barbara. B. Moments clés — Yova détecte et affiche des cartes ponctuelles ("Barbara a géré 5 tâches enfants cette semaine — 2× la moyenne"). 1-2 cartes/sem max, qualité &gt; quantité.</v>
       </c>
       <c r="D3" t="str">
         <v>À faire</v>
       </c>
       <c r="E3" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F3" t="str">
-        <v/>
+        <v>Post-tests Barbara</v>
       </c>
     </row>
     <row r="4">
@@ -996,19 +996,19 @@
         <v>2.3</v>
       </c>
       <c r="B4" t="str">
-        <v>Wire up /api/ai/weekly-summary</v>
+        <v>Détection de routines</v>
       </c>
       <c r="C4" t="str">
-        <v>Version IA enrichie du récap dimanche (actuellement stats pures côté client). Remplacer la carte récap dans /journal par appel Claude.</v>
+        <v>Yova observe : si tâches A+B+C complétées ensemble (même 2h, même personne, ≥3 fois), propose "Je regroupe en routine X ? 1 tap = les 3 marquées faites." Nouvelle table task_routines. Gain friction massif pour les routines quotidiennes (soir enfants, matin école).</v>
       </c>
       <c r="D4" t="str">
         <v>À faire</v>
       </c>
       <c r="E4" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F4" t="str">
-        <v/>
+        <v>Post-tests Barbara</v>
       </c>
     </row>
     <row r="5">
@@ -1016,10 +1016,10 @@
         <v>2.4</v>
       </c>
       <c r="B5" t="str">
-        <v>UX subtasks : refiner</v>
+        <v>SMS hebdo au partenaire non-installé</v>
       </c>
       <c r="C5" t="str">
-        <v>La décomposition auto est active. Tester le comportement sur 5-10 tâches variées. Ajuster le seuil de Claude (3+ sous-tâches min). Ajouter analytics : combien de fois l'écran s'affiche, combien sont créées vs passées.</v>
+        <v>Option d'invitation : user saisit nº téléphone partenaire, SMS opt-in RGPD-compliant ("réponds OUI/STOP"). Si OUI, SMS dimanche soir résumant la semaine reconnue. Canal social léger sans forcer l'install.</v>
       </c>
       <c r="D5" t="str">
         <v>À faire</v>
@@ -1028,7 +1028,7 @@
         <v>P2</v>
       </c>
       <c r="F5" t="str">
-        <v/>
+        <v>RGPD clause à rédiger dans CGU</v>
       </c>
     </row>
     <row r="6">
@@ -1036,24 +1036,84 @@
         <v>2.5</v>
       </c>
       <c r="B6" t="str">
-        <v>Présenter subtasks dans /tasks/catalog</v>
+        <v>Wire up /api/ai/anticipate</v>
       </c>
       <c r="C6" t="str">
-        <v>Quand un template est ajouté via catalogue, vérifier que la décomposition auto se déclenche aussi (pas seulement via /tasks/new).</v>
+        <v>Endpoint d'anticipation proactive (tâches à venir, rappels). Route existe côté serveur. Brancher au Journal : Yova mentionne proactivement les tâches qui arrivent cette semaine.</v>
       </c>
       <c r="D6" t="str">
         <v>À faire</v>
       </c>
       <c r="E6" t="str">
+        <v>P1</v>
+      </c>
+      <c r="F6" t="str">
+        <v>User insistait dessus</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>2.6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Wire up /api/ai/insights</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Insights IA hebdomadaires (version Premium de ce que DashboardFree fait côté client). Brancher au dashboard derrière gate Premium.</v>
+      </c>
+      <c r="D7" t="str">
+        <v>À faire</v>
+      </c>
+      <c r="E7" t="str">
         <v>P2</v>
       </c>
-      <c r="F6" t="str">
+      <c r="F7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>2.7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Wire up /api/ai/weekly-summary</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Version IA enrichie du récap dimanche (actuellement stats pures côté client). Remplacer la carte récap dans /journal par appel Claude.</v>
+      </c>
+      <c r="D8" t="str">
+        <v>À faire</v>
+      </c>
+      <c r="E8" t="str">
+        <v>P2</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>2.8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>UX subtasks : refiner</v>
+      </c>
+      <c r="C9" t="str">
+        <v>La décomposition auto est active. Tester le comportement sur 5-10 tâches variées. Ajuster le seuil de Claude (3+ sous-tâches min). Ajouter analytics : combien de fois l'écran s'affiche, combien sont créées vs passées.</v>
+      </c>
+      <c r="D9" t="str">
+        <v>À faire</v>
+      </c>
+      <c r="E9" t="str">
+        <v>P2</v>
+      </c>
+      <c r="F9" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>